<commit_message>
Update absensi 25 Mei 2026 - PG, TKB2, TKB1, TKa
</commit_message>
<xml_diff>
--- a/PC-06/docs/ABSENSI Mei.xlsx
+++ b/PC-06/docs/ABSENSI Mei.xlsx
@@ -1153,7 +1153,11 @@
       <c r="Y7" s="8" t="n"/>
       <c r="Z7" s="8" t="n"/>
       <c r="AA7" s="8" t="n"/>
-      <c r="AB7" s="8" t="n"/>
+      <c r="AB7" s="8" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
       <c r="AC7" s="8" t="n"/>
       <c r="AD7" s="8" t="n"/>
       <c r="AE7" s="8" t="n"/>
@@ -1248,9 +1252,21 @@
       <c r="R9" s="8" t="n"/>
       <c r="S9" s="8" t="n"/>
       <c r="T9" s="8" t="n"/>
-      <c r="U9" s="8" t="n"/>
-      <c r="V9" s="8" t="n"/>
-      <c r="W9" s="8" t="n"/>
+      <c r="U9" s="8" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="V9" s="8" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="W9" s="8" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
       <c r="X9" s="8" t="n"/>
       <c r="Y9" s="8" t="n"/>
       <c r="Z9" s="8" t="n"/>
@@ -1302,7 +1318,11 @@
       <c r="U10" s="12" t="n"/>
       <c r="V10" s="12" t="n"/>
       <c r="W10" s="12" t="n"/>
-      <c r="X10" s="12" t="n"/>
+      <c r="X10" s="12" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
       <c r="Y10" s="12" t="n"/>
       <c r="Z10" s="12" t="n"/>
       <c r="AA10" s="12" t="n"/>
@@ -1403,7 +1423,11 @@
       <c r="U12" s="8" t="n"/>
       <c r="V12" s="8" t="n"/>
       <c r="W12" s="8" t="n"/>
-      <c r="X12" s="8" t="n"/>
+      <c r="X12" s="8" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
       <c r="Y12" s="8" t="n"/>
       <c r="Z12" s="8" t="n"/>
       <c r="AA12" s="8" t="n"/>
@@ -5204,7 +5228,11 @@
       <c r="T21" s="8" t="n"/>
       <c r="U21" s="8" t="n"/>
       <c r="V21" s="8" t="n"/>
-      <c r="W21" s="8" t="n"/>
+      <c r="W21" s="8" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
       <c r="X21" s="8" t="n"/>
       <c r="Y21" s="8" t="n"/>
       <c r="Z21" s="8" t="n"/>
@@ -5305,7 +5333,11 @@
       <c r="Y23" s="8" t="n"/>
       <c r="Z23" s="8" t="n"/>
       <c r="AA23" s="8" t="n"/>
-      <c r="AB23" s="8" t="n"/>
+      <c r="AB23" s="8" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
       <c r="AC23" s="8" t="n"/>
       <c r="AD23" s="8" t="n"/>
       <c r="AE23" s="8" t="n"/>
@@ -5593,7 +5625,11 @@
       <c r="Y29" s="8" t="n"/>
       <c r="Z29" s="8" t="n"/>
       <c r="AA29" s="8" t="n"/>
-      <c r="AB29" s="8" t="n"/>
+      <c r="AB29" s="8" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
       <c r="AC29" s="8" t="n"/>
       <c r="AD29" s="8" t="n"/>
       <c r="AE29" s="8" t="n"/>
@@ -5683,9 +5719,21 @@
       <c r="S31" s="8" t="n"/>
       <c r="T31" s="8" t="n"/>
       <c r="U31" s="8" t="n"/>
-      <c r="V31" s="8" t="n"/>
-      <c r="W31" s="8" t="n"/>
-      <c r="X31" s="8" t="n"/>
+      <c r="V31" s="8" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="W31" s="8" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="X31" s="8" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
       <c r="Y31" s="8" t="n"/>
       <c r="Z31" s="8" t="n"/>
       <c r="AA31" s="8" t="n"/>
@@ -5875,7 +5923,11 @@
       <c r="S35" s="8" t="n"/>
       <c r="T35" s="8" t="n"/>
       <c r="U35" s="8" t="n"/>
-      <c r="V35" s="8" t="n"/>
+      <c r="V35" s="8" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
       <c r="W35" s="8" t="n"/>
       <c r="X35" s="8" t="n"/>
       <c r="Y35" s="8" t="n"/>
@@ -7495,7 +7547,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AO55"/>
+  <dimension ref="A1:AW55"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="14.453125" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="6.453125" customWidth="1" style="36" min="1" max="1"/>
@@ -8768,7 +8820,11 @@
       <c r="S24" s="8" t="n"/>
       <c r="T24" s="8" t="n"/>
       <c r="U24" s="8" t="n"/>
-      <c r="V24" s="8" t="n"/>
+      <c r="V24" s="8" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
       <c r="W24" s="8" t="n"/>
       <c r="X24" s="8" t="n"/>
       <c r="Y24" s="8" t="n"/>
@@ -9306,7 +9362,11 @@
       <c r="Y35" s="8" t="n"/>
       <c r="Z35" s="8" t="n"/>
       <c r="AA35" s="8" t="n"/>
-      <c r="AB35" s="8" t="n"/>
+      <c r="AB35" s="8" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
       <c r="AC35" s="8" t="n"/>
       <c r="AD35" s="8" t="n"/>
       <c r="AE35" s="8" t="n"/>
@@ -9354,7 +9414,11 @@
       <c r="Y36" s="8" t="n"/>
       <c r="Z36" s="8" t="n"/>
       <c r="AA36" s="8" t="n"/>
-      <c r="AB36" s="8" t="n"/>
+      <c r="AB36" s="8" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
       <c r="AC36" s="8" t="n"/>
       <c r="AD36" s="8" t="n"/>
       <c r="AE36" s="8" t="n"/>
@@ -11553,9 +11617,17 @@
       <c r="S10" s="8" t="n"/>
       <c r="T10" s="8" t="n"/>
       <c r="U10" s="8" t="n"/>
-      <c r="V10" s="8" t="n"/>
+      <c r="V10" s="8" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
       <c r="W10" s="8" t="n"/>
-      <c r="X10" s="8" t="n"/>
+      <c r="X10" s="8" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
       <c r="Y10" s="8" t="n"/>
       <c r="Z10" s="8" t="n"/>
       <c r="AA10" s="8" t="n"/>
@@ -12034,13 +12106,21 @@
       <c r="S20" s="8" t="n"/>
       <c r="T20" s="8" t="n"/>
       <c r="U20" s="8" t="n"/>
-      <c r="V20" s="8" t="n"/>
+      <c r="V20" s="8" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
       <c r="W20" s="8" t="n"/>
       <c r="X20" s="8" t="n"/>
       <c r="Y20" s="8" t="n"/>
       <c r="Z20" s="8" t="n"/>
       <c r="AA20" s="8" t="n"/>
-      <c r="AB20" s="8" t="n"/>
+      <c r="AB20" s="8" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
       <c r="AC20" s="8" t="n"/>
       <c r="AD20" s="8" t="n"/>
       <c r="AE20" s="8" t="n"/>
@@ -12227,7 +12307,11 @@
       <c r="T24" s="8" t="n"/>
       <c r="U24" s="8" t="n"/>
       <c r="V24" s="8" t="n"/>
-      <c r="W24" s="8" t="n"/>
+      <c r="W24" s="8" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
       <c r="X24" s="8" t="n"/>
       <c r="Y24" s="8" t="n"/>
       <c r="Z24" s="8" t="n"/>
@@ -12418,7 +12502,11 @@
       <c r="S28" s="8" t="n"/>
       <c r="T28" s="8" t="n"/>
       <c r="U28" s="8" t="n"/>
-      <c r="V28" s="8" t="n"/>
+      <c r="V28" s="8" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
       <c r="W28" s="8" t="n"/>
       <c r="X28" s="8" t="n"/>
       <c r="Y28" s="8" t="n"/>
@@ -12708,7 +12796,11 @@
       <c r="U34" s="8" t="n"/>
       <c r="V34" s="8" t="n"/>
       <c r="W34" s="8" t="n"/>
-      <c r="X34" s="8" t="n"/>
+      <c r="X34" s="8" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
       <c r="Y34" s="8" t="n"/>
       <c r="Z34" s="8" t="n"/>
       <c r="AA34" s="8" t="n"/>

</xml_diff>